<commit_message>
Fix Example 4 sample data — proper NPS ratings and renamed score column
create_sample_data.py:
- nps_score now generates 0–10 raw survey ratings (Promoters 9–10,
  Passives 7–8, Detractors 0–6) instead of pre-computed 20–72 values
- Inactive accounts in Period 2 pull down to Detractor range (0–6)
  so the NPS Promoter/Passive/Detractor breakdown shows a real change
- Renamed "score" column to "account_health_score" so the LLM has a
  meaningful name to use in explanations (not just "score")

Sample data regenerated for all 4 examples.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/example4_mixed/Mixed_april_2025.xlsx
+++ b/sample_data/example4_mixed/Mixed_april_2025.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>score</t>
+          <t>account_health_score</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -491,7 +491,7 @@
         <v>63</v>
       </c>
       <c r="G2" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -520,7 +520,7 @@
         <v>74</v>
       </c>
       <c r="G3" t="n">
-        <v>62</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         <v>73</v>
       </c>
       <c r="G4" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -578,7 +578,7 @@
         <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -607,7 +607,7 @@
         <v>78</v>
       </c>
       <c r="G6" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -636,7 +636,7 @@
         <v>87</v>
       </c>
       <c r="G7" t="n">
-        <v>49</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -665,7 +665,7 @@
         <v>93</v>
       </c>
       <c r="G8" t="n">
-        <v>53</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -694,7 +694,7 @@
         <v>68</v>
       </c>
       <c r="G9" t="n">
-        <v>71</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -723,7 +723,7 @@
         <v>91</v>
       </c>
       <c r="G10" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -752,7 +752,7 @@
         <v>91</v>
       </c>
       <c r="G11" t="n">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -781,7 +781,7 @@
         <v>95</v>
       </c>
       <c r="G12" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -810,7 +810,7 @@
         <v>70</v>
       </c>
       <c r="G13" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -839,7 +839,7 @@
         <v>89</v>
       </c>
       <c r="G14" t="n">
-        <v>68</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -868,7 +868,7 @@
         <v>78</v>
       </c>
       <c r="G15" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -897,7 +897,7 @@
         <v>57</v>
       </c>
       <c r="G16" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -926,7 +926,7 @@
         <v>66</v>
       </c>
       <c r="G17" t="n">
-        <v>41</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18">
@@ -955,7 +955,7 @@
         <v>82</v>
       </c>
       <c r="G18" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -984,7 +984,7 @@
         <v>61</v>
       </c>
       <c r="G19" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -1013,7 +1013,7 @@
         <v>72</v>
       </c>
       <c r="G20" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -1042,7 +1042,7 @@
         <v>86</v>
       </c>
       <c r="G21" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -1071,7 +1071,7 @@
         <v>61</v>
       </c>
       <c r="G22" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -1100,7 +1100,7 @@
         <v>75</v>
       </c>
       <c r="G23" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -1129,7 +1129,7 @@
         <v>63</v>
       </c>
       <c r="G24" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -1158,7 +1158,7 @@
         <v>76</v>
       </c>
       <c r="G25" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
@@ -1187,7 +1187,7 @@
         <v>64</v>
       </c>
       <c r="G26" t="n">
-        <v>56</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27">
@@ -1216,7 +1216,7 @@
         <v>94</v>
       </c>
       <c r="G27" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -1245,7 +1245,7 @@
         <v>58</v>
       </c>
       <c r="G28" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29">
@@ -1274,7 +1274,7 @@
         <v>94</v>
       </c>
       <c r="G29" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30">
@@ -1303,7 +1303,7 @@
         <v>87</v>
       </c>
       <c r="G30" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31">
@@ -1332,7 +1332,7 @@
         <v>90</v>
       </c>
       <c r="G31" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
@@ -1361,7 +1361,7 @@
         <v>89</v>
       </c>
       <c r="G32" t="n">
-        <v>68</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33">
@@ -1390,7 +1390,7 @@
         <v>62</v>
       </c>
       <c r="G33" t="n">
-        <v>47</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34">
@@ -1419,7 +1419,7 @@
         <v>93</v>
       </c>
       <c r="G34" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -1448,7 +1448,7 @@
         <v>79</v>
       </c>
       <c r="G35" t="n">
-        <v>44</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36">
@@ -1477,7 +1477,7 @@
         <v>94</v>
       </c>
       <c r="G36" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37">
@@ -1506,7 +1506,7 @@
         <v>91</v>
       </c>
       <c r="G37" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38">
@@ -1535,7 +1535,7 @@
         <v>78</v>
       </c>
       <c r="G38" t="n">
-        <v>50</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39">
@@ -1564,7 +1564,7 @@
         <v>70</v>
       </c>
       <c r="G39" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40">
@@ -1593,7 +1593,7 @@
         <v>59</v>
       </c>
       <c r="G40" t="n">
-        <v>52</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41">
@@ -1622,7 +1622,7 @@
         <v>59</v>
       </c>
       <c r="G41" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>